<commit_message>
docs(examples): add excel detection payload example
</commit_message>
<xml_diff>
--- a/examples/detection/excel/excel_addresses_example.xlsx
+++ b/examples/detection/excel/excel_addresses_example.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/afryan/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/afryan/IdeaProjects/geo-jobs/examples/detection/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1DEE377-149D-B640-9975-00F024C0CEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B794E0D5-4DD0-8242-849A-CA8599C7CE0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{5579C3DA-00F9-424E-B5A9-3EA9B5569F70}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="181029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,7 +38,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
-    <t>238 Rue Pierre Mauroy</t>
+    <t>8 Rue Stephen Liegeard, 06400 Cannes, France</t>
   </si>
 </sst>
 </file>

</xml_diff>